<commit_message>
chore: Update template and mapping files
</commit_message>
<xml_diff>
--- a/Template/Template SO - PO.xlsx
+++ b/Template/Template SO - PO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://my.maerskgroup.com/personal/phuong_chung_maersk_com/Documents/Desktop/OBOUND/Tháng 6/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\AI Learning\Generate ASN\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1814" documentId="13_ncr:1_{1681AB3D-3F75-4173-9E3B-7781DB98F501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F97A062D-ABD3-47BB-B257-272EE48F48F7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E3A4C0F-15B4-4833-A1FC-7A4D9FB67B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -257,7 +257,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t>ExternOrderkey</t>
   </si>
@@ -890,57 +890,6 @@
   </si>
   <si>
     <t>TariffKey</t>
-  </si>
-  <si>
-    <t>DANONE</t>
-  </si>
-  <si>
-    <t>DAN1_SO</t>
-  </si>
-  <si>
-    <t>Loose</t>
-  </si>
-  <si>
-    <t>DAN1</t>
-  </si>
-  <si>
-    <t>EA</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>AB</t>
-  </si>
-  <si>
-    <t>2028.02.10</t>
-  </si>
-  <si>
-    <t>PO2-0626_T1</t>
-  </si>
-  <si>
-    <t>PO2-0626_T2</t>
-  </si>
-  <si>
-    <t>HoangLe_HCM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lô M7-M9-M11, Đường A, </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> phường Cát Lái, TP.HCM</t>
-  </si>
-  <si>
-    <t>South</t>
-  </si>
-  <si>
-    <t>2028.02.25</t>
-  </si>
-  <si>
-    <t>2028.03.06</t>
-  </si>
-  <si>
-    <t>C</t>
   </si>
 </sst>
 </file>
@@ -2114,301 +2063,21 @@
       </c>
     </row>
     <row r="2" spans="1:211" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B2" t="s">
-        <v>211</v>
-      </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="2">
-        <v>46179</v>
-      </c>
-      <c r="G2" t="s">
-        <v>221</v>
-      </c>
-      <c r="J2" t="s">
-        <v>221</v>
-      </c>
-      <c r="K2" t="s">
-        <v>222</v>
-      </c>
-      <c r="L2" t="s">
-        <v>223</v>
-      </c>
-      <c r="P2" t="s">
-        <v>224</v>
-      </c>
-      <c r="AZ2" t="s">
-        <v>212</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>213</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>214</v>
-      </c>
-      <c r="BT2">
-        <v>43785558</v>
-      </c>
-      <c r="CO2">
-        <v>1</v>
-      </c>
-      <c r="CP2">
-        <v>194403</v>
-      </c>
+      <c r="E2" s="2"/>
       <c r="CV2" s="4"/>
-      <c r="CW2">
-        <v>6090</v>
-      </c>
-      <c r="CX2" t="s">
-        <v>215</v>
-      </c>
-      <c r="DG2" t="s">
-        <v>225</v>
-      </c>
-      <c r="DH2" t="s">
-        <v>217</v>
-      </c>
-      <c r="FK2" t="s">
-        <v>216</v>
-      </c>
     </row>
     <row r="3" spans="1:211" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>219</v>
-      </c>
-      <c r="B3" t="s">
-        <v>211</v>
-      </c>
-      <c r="E3" s="2">
-        <v>46179</v>
-      </c>
-      <c r="G3" t="s">
-        <v>221</v>
-      </c>
-      <c r="J3" t="s">
-        <v>221</v>
-      </c>
-      <c r="K3" t="s">
-        <v>222</v>
-      </c>
-      <c r="L3" t="s">
-        <v>223</v>
-      </c>
-      <c r="P3" t="s">
-        <v>224</v>
-      </c>
-      <c r="AZ3" t="s">
-        <v>212</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>213</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>214</v>
-      </c>
-      <c r="BT3">
-        <v>43785558</v>
-      </c>
-      <c r="CO3">
-        <v>2</v>
-      </c>
-      <c r="CP3">
-        <v>194403</v>
-      </c>
-      <c r="CW3">
-        <v>153</v>
-      </c>
-      <c r="CX3" t="s">
-        <v>215</v>
-      </c>
-      <c r="DG3" t="s">
-        <v>225</v>
-      </c>
-      <c r="DH3" t="s">
-        <v>227</v>
-      </c>
-      <c r="FK3" t="s">
-        <v>216</v>
-      </c>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:211" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>219</v>
-      </c>
-      <c r="B4" t="s">
-        <v>211</v>
-      </c>
-      <c r="E4" s="2">
-        <v>46179</v>
-      </c>
-      <c r="G4" t="s">
-        <v>221</v>
-      </c>
-      <c r="J4" t="s">
-        <v>221</v>
-      </c>
-      <c r="K4" t="s">
-        <v>222</v>
-      </c>
-      <c r="L4" t="s">
-        <v>223</v>
-      </c>
-      <c r="P4" t="s">
-        <v>224</v>
-      </c>
-      <c r="AZ4" t="s">
-        <v>212</v>
-      </c>
-      <c r="BE4" t="s">
-        <v>213</v>
-      </c>
-      <c r="BQ4" t="s">
-        <v>214</v>
-      </c>
-      <c r="BT4">
-        <v>43785558</v>
-      </c>
-      <c r="CO4">
-        <v>3</v>
-      </c>
-      <c r="CP4">
-        <v>194404</v>
-      </c>
-      <c r="CW4">
-        <v>228</v>
-      </c>
-      <c r="CX4" t="s">
-        <v>215</v>
-      </c>
-      <c r="DG4" t="s">
-        <v>218</v>
-      </c>
-      <c r="DH4" t="s">
-        <v>227</v>
-      </c>
-      <c r="FK4" t="s">
-        <v>216</v>
-      </c>
+      <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:211" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>219</v>
-      </c>
-      <c r="B5" t="s">
-        <v>211</v>
-      </c>
-      <c r="E5" s="2">
-        <v>46179</v>
-      </c>
-      <c r="G5" t="s">
-        <v>221</v>
-      </c>
-      <c r="J5" t="s">
-        <v>221</v>
-      </c>
-      <c r="K5" t="s">
-        <v>222</v>
-      </c>
-      <c r="L5" t="s">
-        <v>223</v>
-      </c>
-      <c r="P5" t="s">
-        <v>224</v>
-      </c>
-      <c r="AZ5" t="s">
-        <v>212</v>
-      </c>
-      <c r="BE5" t="s">
-        <v>213</v>
-      </c>
-      <c r="BQ5" t="s">
-        <v>214</v>
-      </c>
-      <c r="BT5">
-        <v>43785558</v>
-      </c>
-      <c r="CO5">
-        <v>4</v>
-      </c>
-      <c r="CP5">
-        <v>194405</v>
-      </c>
-      <c r="CW5">
-        <v>542</v>
-      </c>
-      <c r="CX5" t="s">
-        <v>215</v>
-      </c>
-      <c r="DG5" t="s">
-        <v>226</v>
-      </c>
-      <c r="DH5" t="s">
-        <v>227</v>
-      </c>
-      <c r="FK5" t="s">
-        <v>216</v>
-      </c>
+      <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:211" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>220</v>
-      </c>
-      <c r="B6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E6" s="2">
-        <v>46179</v>
-      </c>
-      <c r="G6" t="s">
-        <v>221</v>
-      </c>
-      <c r="J6" t="s">
-        <v>221</v>
-      </c>
-      <c r="K6" t="s">
-        <v>222</v>
-      </c>
-      <c r="L6" t="s">
-        <v>223</v>
-      </c>
-      <c r="P6" t="s">
-        <v>224</v>
-      </c>
-      <c r="AZ6" t="s">
-        <v>212</v>
-      </c>
-      <c r="BE6" t="s">
-        <v>213</v>
-      </c>
-      <c r="BQ6" t="s">
-        <v>214</v>
-      </c>
-      <c r="BT6">
-        <v>43785558</v>
-      </c>
-      <c r="CO6">
-        <v>5</v>
-      </c>
-      <c r="CP6">
-        <v>194404</v>
-      </c>
-      <c r="CW6">
-        <v>420</v>
-      </c>
-      <c r="CX6" t="s">
-        <v>215</v>
-      </c>
-      <c r="DG6" t="s">
-        <v>218</v>
-      </c>
-      <c r="DH6" t="s">
-        <v>217</v>
-      </c>
-      <c r="FK6" t="s">
-        <v>216</v>
-      </c>
+      <c r="E6" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:HC2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
@@ -2437,6 +2106,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007302575D815E474FB4FB92317EDADB55" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="65c82f07a89316cf344e67860d3a10d3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="44026def-ea23-43d6-bb21-f57ce08e746f" xmlns:ns3="36837cc5-0ce9-4798-aec4-1237aab959ef" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4441ee74b6b3fc1c3454b40309a894b7" ns2:_="" ns3:_="">
     <xsd:import namespace="44026def-ea23-43d6-bb21-f57ce08e746f"/>
@@ -2705,15 +2383,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3329D120-3361-4628-9312-CFEB2C65925D}">
   <ds:schemaRefs>
@@ -2726,6 +2395,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EC8C2AE-7BFC-455B-ADDE-48CC0A1BA54E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B75E6C6-D6F5-4BF5-9F52-C569B0807112}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2742,12 +2419,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EC8C2AE-7BFC-455B-ADDE-48CC0A1BA54E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>